<commit_message>
Maintenance workflow v2: parts-check scheduling, smart todo, inventory intake, and parts/location management
</commit_message>
<xml_diff>
--- a/maintenance/BottomCenteringPulley_BreakDetector_Maintenance_Tracker_Template.xlsx
+++ b/maintenance/BottomCenteringPulley_BreakDetector_Maintenance_Tracker_Template.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,26 @@
           <t>Last Done Furnace Hours</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Required Parts</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Planning months</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Estimated duration min</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -613,6 +633,18 @@
       <c r="T2" t="n">
         <v>0</v>
       </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Routine</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -696,6 +728,22 @@
       </c>
       <c r="T3" t="n">
         <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Bearing set; IPA wipes / cleaning cloth</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X3" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WIP: checkpoint maintenance auto flow baseline
</commit_message>
<xml_diff>
--- a/maintenance/BottomCenteringPulley_BreakDetector_Maintenance_Tracker_Template.xlsx
+++ b/maintenance/BottomCenteringPulley_BreakDetector_Maintenance_Tracker_Template.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,22 +531,47 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Required Parts</t>
+          <t>Required_Parts</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Task_Group</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Planning months</t>
+          <t>Planning_Window_Months</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Estimated duration min</t>
+          <t>Est_Duration_Min</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Last_Done_Draw</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Task_Groups</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Last_Done_Hours_UV1</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Last_Done_Hours_UV2</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Last_Done_Hours_Furnace</t>
         </is>
       </c>
     </row>
@@ -589,7 +614,6 @@
           <t>calendar</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>months</t>
@@ -621,22 +645,17 @@
           <t>Working at height: stay behind guard rails and/or use safety harness; good housekeeping to prevent dropped items.</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2025-01-22</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
+          <t>2026-02-26</t>
+        </is>
       </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
-      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Routine</t>
+          <t>3-Month</t>
         </is>
       </c>
       <c r="W2" t="n">
@@ -644,6 +663,11 @@
       </c>
       <c r="X2" t="n">
         <v>20</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>3-Month</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -685,7 +709,6 @@
           <t>calendar</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>weeks</t>
@@ -717,14 +740,10 @@
           <t>Methanol is toxic and can be absorbed through skin on prolonged exposure; wear impermeable gloves.</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2025-01-22</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
+          <t>2026-03-29</t>
+        </is>
       </c>
       <c r="T3" t="n">
         <v>0</v>

</xml_diff>